<commit_message>
feat: translate UI to French, add extraction log, handle Commande Tissu, and improve OCR detection
</commit_message>
<xml_diff>
--- a/out/output.xlsx
+++ b/out/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
   <si>
     <t>OrderNumber</t>
   </si>
@@ -37,6 +37,48 @@
     <t>Size</t>
   </si>
   <si>
+    <t>0000.04031</t>
+  </si>
+  <si>
+    <t>1/0/1</t>
+  </si>
+  <si>
+    <t>11887</t>
+  </si>
+  <si>
+    <t>ZICHT</t>
+  </si>
+  <si>
+    <t>OFF251665 - Kamila Zareba</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>730.8 x 261.5</t>
+  </si>
+  <si>
+    <t>0000.04032</t>
+  </si>
+  <si>
+    <t>1/1/1</t>
+  </si>
+  <si>
+    <t>05561</t>
+  </si>
+  <si>
+    <t>MEGA MEUBEL</t>
+  </si>
+  <si>
+    <t>Olga</t>
+  </si>
+  <si>
+    <t>127 x 225</t>
+  </si>
+  <si>
+    <t>1/2/1</t>
+  </si>
+  <si>
     <t>0000.04033</t>
   </si>
   <si>
@@ -100,12 +142,225 @@
     <t>6/2/6</t>
   </si>
   <si>
+    <t>0000.04034</t>
+  </si>
+  <si>
+    <t>1/0/36</t>
+  </si>
+  <si>
+    <t>12024</t>
+  </si>
+  <si>
+    <t>The Marketing Collective B.V.</t>
+  </si>
+  <si>
+    <t>mail 25/02</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>2/0/36</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>3/0/36</t>
+  </si>
+  <si>
+    <t>4/0/36</t>
+  </si>
+  <si>
+    <t>5/0/36</t>
+  </si>
+  <si>
+    <t>6/0/36</t>
+  </si>
+  <si>
+    <t>7/0/36</t>
+  </si>
+  <si>
+    <t>8/0/36</t>
+  </si>
+  <si>
+    <t>9/0/36</t>
+  </si>
+  <si>
+    <t>10/0/36</t>
+  </si>
+  <si>
+    <t>11/0/36</t>
+  </si>
+  <si>
+    <t>12/0/36</t>
+  </si>
+  <si>
+    <t>13/0/36</t>
+  </si>
+  <si>
+    <t>14/0/36</t>
+  </si>
+  <si>
+    <t>15/0/36</t>
+  </si>
+  <si>
+    <t>16/0/36</t>
+  </si>
+  <si>
+    <t>17/0/36</t>
+  </si>
+  <si>
+    <t>18/0/36</t>
+  </si>
+  <si>
+    <t>19/0/36</t>
+  </si>
+  <si>
+    <t>20/0/36</t>
+  </si>
+  <si>
+    <t>21/0/36</t>
+  </si>
+  <si>
+    <t>22/0/36</t>
+  </si>
+  <si>
+    <t>23/0/36</t>
+  </si>
+  <si>
+    <t>24/0/36</t>
+  </si>
+  <si>
+    <t>25/0/36</t>
+  </si>
+  <si>
+    <t>26/0/36</t>
+  </si>
+  <si>
+    <t>27/0/36</t>
+  </si>
+  <si>
+    <t>28/0/36</t>
+  </si>
+  <si>
+    <t>29/0/36</t>
+  </si>
+  <si>
+    <t>30/0/36</t>
+  </si>
+  <si>
+    <t>31/0/36</t>
+  </si>
+  <si>
+    <t>32/0/36</t>
+  </si>
+  <si>
+    <t>33/0/36</t>
+  </si>
+  <si>
+    <t>34/0/36</t>
+  </si>
+  <si>
+    <t>35/0/36</t>
+  </si>
+  <si>
+    <t>36/0/36</t>
+  </si>
+  <si>
+    <t>601L.00293</t>
+  </si>
+  <si>
+    <t>1/1/2</t>
+  </si>
+  <si>
+    <t>02592</t>
+  </si>
+  <si>
+    <t>HISTOIRES D'OMBRES</t>
+  </si>
+  <si>
+    <t>L0102 SAMANIEGO</t>
+  </si>
+  <si>
+    <t>Fenêtre G</t>
+  </si>
+  <si>
+    <t>105 x 173.5</t>
+  </si>
+  <si>
+    <t>1/2/2</t>
+  </si>
+  <si>
+    <t>125 x 173.5</t>
+  </si>
+  <si>
+    <t>2/1/2</t>
+  </si>
+  <si>
+    <t>Fenêtre D</t>
+  </si>
+  <si>
+    <t>95 x 173.5</t>
+  </si>
+  <si>
+    <t>2/2/2</t>
+  </si>
+  <si>
+    <t>70 x 173.5</t>
+  </si>
+  <si>
+    <t>603Z.00041</t>
+  </si>
+  <si>
+    <t>1/0/2</t>
+  </si>
+  <si>
+    <t>05381</t>
+  </si>
+  <si>
+    <t>RULOT HOME DECORATION SA</t>
+  </si>
+  <si>
+    <t>Magonnette</t>
+  </si>
+  <si>
+    <t>séjour baie d'angle</t>
+  </si>
+  <si>
+    <t>179 x 253</t>
+  </si>
+  <si>
+    <t>2/0/2</t>
+  </si>
+  <si>
+    <t>Séjour pignon</t>
+  </si>
+  <si>
+    <t>220.5 x 253.5</t>
+  </si>
+  <si>
+    <t>60AZ.00333</t>
+  </si>
+  <si>
+    <t>07196</t>
+  </si>
+  <si>
+    <t>CORTINA</t>
+  </si>
+  <si>
+    <t>Sanen</t>
+  </si>
+  <si>
+    <t>woonkamer</t>
+  </si>
+  <si>
+    <t>430 x 246</t>
+  </si>
+  <si>
     <t>60CW.00058</t>
   </si>
   <si>
-    <t>1/0/2</t>
-  </si>
-  <si>
     <t>03490</t>
   </si>
   <si>
@@ -119,9 +374,6 @@
   </si>
   <si>
     <t>170 x 256</t>
-  </si>
-  <si>
-    <t>2/0/2</t>
   </si>
   <si>
     <t>345 x 256</t>
@@ -434,9 +686,10 @@
     <col customWidth="true" max="1" min="1" width="13"/>
     <col customWidth="true" max="2" min="2" width="11"/>
     <col customWidth="true" max="3" min="3" width="12"/>
-    <col customWidth="true" max="4" min="4" width="17"/>
-    <col customWidth="true" max="5" min="5" width="15"/>
-    <col customWidth="true" max="7" min="6" width="11"/>
+    <col customWidth="true" max="4" min="4" width="31"/>
+    <col customWidth="true" max="5" min="5" width="27"/>
+    <col customWidth="true" max="6" min="6" width="22"/>
+    <col customWidth="true" max="7" min="7" width="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,301 +740,1359 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
         <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G6" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
         <v>25</v>
       </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
       <c r="F10" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G10" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="F13" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G13" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G14" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="G15" t="s">
-        <v>36</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" t="s">
+        <v>46</v>
+      </c>
+      <c r="F23" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" t="s">
+        <v>46</v>
+      </c>
+      <c r="F24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" t="s">
+        <v>46</v>
+      </c>
+      <c r="F25" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" t="s">
+        <v>46</v>
+      </c>
+      <c r="F26" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" t="s">
+        <v>46</v>
+      </c>
+      <c r="F27" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28" t="s">
+        <v>46</v>
+      </c>
+      <c r="F28" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" t="s">
+        <v>46</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" t="s">
+        <v>45</v>
+      </c>
+      <c r="E30" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" t="s">
+        <v>45</v>
+      </c>
+      <c r="E33" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" t="s">
+        <v>45</v>
+      </c>
+      <c r="E34" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E35" t="s">
+        <v>46</v>
+      </c>
+      <c r="F35" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" t="s">
+        <v>44</v>
+      </c>
+      <c r="D36" t="s">
+        <v>45</v>
+      </c>
+      <c r="E36" t="s">
+        <v>46</v>
+      </c>
+      <c r="F36" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" t="s">
+        <v>70</v>
+      </c>
+      <c r="C37" t="s">
+        <v>44</v>
+      </c>
+      <c r="D37" t="s">
+        <v>45</v>
+      </c>
+      <c r="E37" t="s">
+        <v>46</v>
+      </c>
+      <c r="F37" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" t="s">
+        <v>44</v>
+      </c>
+      <c r="D38" t="s">
+        <v>45</v>
+      </c>
+      <c r="E38" t="s">
+        <v>46</v>
+      </c>
+      <c r="F38" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" t="s">
+        <v>44</v>
+      </c>
+      <c r="D39" t="s">
+        <v>45</v>
+      </c>
+      <c r="E39" t="s">
+        <v>46</v>
+      </c>
+      <c r="F39" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" t="s">
+        <v>44</v>
+      </c>
+      <c r="D40" t="s">
+        <v>45</v>
+      </c>
+      <c r="E40" t="s">
+        <v>46</v>
+      </c>
+      <c r="F40" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" t="s">
+        <v>44</v>
+      </c>
+      <c r="D41" t="s">
+        <v>45</v>
+      </c>
+      <c r="E41" t="s">
+        <v>46</v>
+      </c>
+      <c r="F41" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D42" t="s">
+        <v>45</v>
+      </c>
+      <c r="E42" t="s">
+        <v>46</v>
+      </c>
+      <c r="F42" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>76</v>
+      </c>
+      <c r="C43" t="s">
+        <v>44</v>
+      </c>
+      <c r="D43" t="s">
+        <v>45</v>
+      </c>
+      <c r="E43" t="s">
+        <v>46</v>
+      </c>
+      <c r="F43" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" t="s">
+        <v>45</v>
+      </c>
+      <c r="E44" t="s">
+        <v>46</v>
+      </c>
+      <c r="F44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" t="s">
+        <v>78</v>
+      </c>
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" t="s">
+        <v>45</v>
+      </c>
+      <c r="E45" t="s">
+        <v>46</v>
+      </c>
+      <c r="F45" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D46" t="s">
+        <v>45</v>
+      </c>
+      <c r="E46" t="s">
+        <v>46</v>
+      </c>
+      <c r="F46" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B47" t="s">
+        <v>80</v>
+      </c>
+      <c r="C47" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" t="s">
+        <v>45</v>
+      </c>
+      <c r="E47" t="s">
+        <v>46</v>
+      </c>
+      <c r="F47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" t="s">
+        <v>81</v>
+      </c>
+      <c r="C48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E48" t="s">
+        <v>46</v>
+      </c>
+      <c r="F48" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>42</v>
+      </c>
+      <c r="B49" t="s">
+        <v>82</v>
+      </c>
+      <c r="C49" t="s">
+        <v>44</v>
+      </c>
+      <c r="D49" t="s">
+        <v>45</v>
+      </c>
+      <c r="E49" t="s">
+        <v>46</v>
+      </c>
+      <c r="F49" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>42</v>
+      </c>
+      <c r="B50" t="s">
+        <v>83</v>
+      </c>
+      <c r="C50" t="s">
+        <v>44</v>
+      </c>
+      <c r="D50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E50" t="s">
+        <v>46</v>
+      </c>
+      <c r="F50" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>84</v>
+      </c>
+      <c r="B51" t="s">
+        <v>85</v>
+      </c>
+      <c r="C51" t="s">
+        <v>86</v>
+      </c>
+      <c r="D51" t="s">
+        <v>87</v>
+      </c>
+      <c r="E51" t="s">
+        <v>88</v>
+      </c>
+      <c r="F51" t="s">
+        <v>89</v>
+      </c>
+      <c r="G51" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>84</v>
+      </c>
+      <c r="B52" t="s">
+        <v>91</v>
+      </c>
+      <c r="C52" t="s">
+        <v>86</v>
+      </c>
+      <c r="D52" t="s">
+        <v>87</v>
+      </c>
+      <c r="E52" t="s">
+        <v>88</v>
+      </c>
+      <c r="F52" t="s">
+        <v>89</v>
+      </c>
+      <c r="G52" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>84</v>
+      </c>
+      <c r="B53" t="s">
+        <v>93</v>
+      </c>
+      <c r="C53" t="s">
+        <v>86</v>
+      </c>
+      <c r="D53" t="s">
+        <v>87</v>
+      </c>
+      <c r="E53" t="s">
+        <v>88</v>
+      </c>
+      <c r="F53" t="s">
+        <v>94</v>
+      </c>
+      <c r="G53" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>84</v>
+      </c>
+      <c r="B54" t="s">
+        <v>96</v>
+      </c>
+      <c r="C54" t="s">
+        <v>86</v>
+      </c>
+      <c r="D54" t="s">
+        <v>87</v>
+      </c>
+      <c r="E54" t="s">
+        <v>88</v>
+      </c>
+      <c r="F54" t="s">
+        <v>94</v>
+      </c>
+      <c r="G54" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>98</v>
+      </c>
+      <c r="B55" t="s">
+        <v>99</v>
+      </c>
+      <c r="C55" t="s">
+        <v>100</v>
+      </c>
+      <c r="D55" t="s">
+        <v>101</v>
+      </c>
+      <c r="E55" t="s">
+        <v>102</v>
+      </c>
+      <c r="F55" t="s">
+        <v>103</v>
+      </c>
+      <c r="G55" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>98</v>
+      </c>
+      <c r="B56" t="s">
+        <v>105</v>
+      </c>
+      <c r="C56" t="s">
+        <v>100</v>
+      </c>
+      <c r="D56" t="s">
+        <v>101</v>
+      </c>
+      <c r="E56" t="s">
+        <v>102</v>
+      </c>
+      <c r="F56" t="s">
+        <v>106</v>
+      </c>
+      <c r="G56" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>108</v>
+      </c>
+      <c r="B57" t="s">
+        <v>8</v>
+      </c>
+      <c r="C57" t="s">
+        <v>109</v>
+      </c>
+      <c r="D57" t="s">
+        <v>110</v>
+      </c>
+      <c r="E57" t="s">
+        <v>111</v>
+      </c>
+      <c r="F57" t="s">
+        <v>112</v>
+      </c>
+      <c r="G57" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>114</v>
+      </c>
+      <c r="B58" t="s">
+        <v>99</v>
+      </c>
+      <c r="C58" t="s">
+        <v>115</v>
+      </c>
+      <c r="D58" t="s">
+        <v>116</v>
+      </c>
+      <c r="E58" t="s">
+        <v>117</v>
+      </c>
+      <c r="F58" t="s">
+        <v>118</v>
+      </c>
+      <c r="G58" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>114</v>
+      </c>
+      <c r="B59" t="s">
+        <v>105</v>
+      </c>
+      <c r="C59" t="s">
+        <v>115</v>
+      </c>
+      <c r="D59" t="s">
+        <v>116</v>
+      </c>
+      <c r="E59" t="s">
+        <v>117</v>
+      </c>
+      <c r="F59" t="s">
+        <v>118</v>
+      </c>
+      <c r="G59" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>114</v>
+      </c>
+      <c r="B60" t="s">
+        <v>99</v>
+      </c>
+      <c r="C60" t="s">
+        <v>115</v>
+      </c>
+      <c r="D60" t="s">
+        <v>116</v>
+      </c>
+      <c r="E60" t="s">
+        <v>117</v>
+      </c>
+      <c r="F60" t="s">
+        <v>118</v>
+      </c>
+      <c r="G60" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>114</v>
+      </c>
+      <c r="B61" t="s">
+        <v>105</v>
+      </c>
+      <c r="C61" t="s">
+        <v>115</v>
+      </c>
+      <c r="D61" t="s">
+        <v>116</v>
+      </c>
+      <c r="E61" t="s">
+        <v>117</v>
+      </c>
+      <c r="F61" t="s">
+        <v>118</v>
+      </c>
+      <c r="G61" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement interactive processing loop in main and update batch script
</commit_message>
<xml_diff>
--- a/out/output.xlsx
+++ b/out/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t>OrderNumber</t>
   </si>
@@ -209,6 +209,60 @@
   </si>
   <si>
     <t>2/0/2</t>
+  </si>
+  <si>
+    <t>60AZ.00344</t>
+  </si>
+  <si>
+    <t>07196</t>
+  </si>
+  <si>
+    <t>CORTINA</t>
+  </si>
+  <si>
+    <t>vermeulen</t>
+  </si>
+  <si>
+    <t>keuken zijraam rechts</t>
+  </si>
+  <si>
+    <t>290 x 270.5</t>
+  </si>
+  <si>
+    <t>keuken zijraam links</t>
+  </si>
+  <si>
+    <t>310 x 270.5</t>
+  </si>
+  <si>
+    <t>3/1/3</t>
+  </si>
+  <si>
+    <t>groot raam gebogen</t>
+  </si>
+  <si>
+    <t>185.0 x 269.5</t>
+  </si>
+  <si>
+    <t>3/2/3</t>
+  </si>
+  <si>
+    <t>0000.04083</t>
+  </si>
+  <si>
+    <t>11676</t>
+  </si>
+  <si>
+    <t>Steef Agenturen</t>
+  </si>
+  <si>
+    <t>stof</t>
+  </si>
+  <si>
+    <t>Monaco</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -521,7 +575,7 @@
     <col customWidth="true" max="4" min="4" width="30"/>
     <col customWidth="true" max="5" min="5" width="11"/>
     <col customWidth="true" max="6" min="6" width="26"/>
-    <col customWidth="true" max="7" min="7" width="13"/>
+    <col customWidth="true" max="7" min="7" width="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -984,6 +1038,121 @@
         <v>63</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F21" t="s">
+        <v>69</v>
+      </c>
+      <c r="G21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" t="s">
+        <v>68</v>
+      </c>
+      <c r="F22" t="s">
+        <v>71</v>
+      </c>
+      <c r="G22" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" t="s">
+        <v>68</v>
+      </c>
+      <c r="F23" t="s">
+        <v>74</v>
+      </c>
+      <c r="G23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" t="s">
+        <v>66</v>
+      </c>
+      <c r="D24" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" t="s">
+        <v>68</v>
+      </c>
+      <c r="F24" t="s">
+        <v>74</v>
+      </c>
+      <c r="G24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" t="s">
+        <v>79</v>
+      </c>
+      <c r="E25" t="s">
+        <v>80</v>
+      </c>
+      <c r="F25" t="s">
+        <v>81</v>
+      </c>
+      <c r="G25" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>